<commit_message>
Extend reusable library with expressions, full-frame layouts and motion
</commit_message>
<xml_diff>
--- a/common_assets/nichijou_naze/management/asset_registry.xlsx
+++ b/common_assets/nichijou_naze/management/asset_registry.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Assets'!$A$1:$K$20</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -413,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1078,7 +1080,448 @@
         <v>1</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>NNZ_CHAR_FEMALE_01</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>キャラ</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>追加表情3種＋V02参照8ポーズ</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>render_verified</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>v03_expressions</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>characters/female_v01/versions/v03_expressions/manifest.json</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>共通素材</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>既存V02参照AI描き起こし＋整形</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>validation/extension/qc-report.json</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>既存V02・旧EP・過去レンダーは不変</t>
+        </is>
+      </c>
+      <c r="K13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>NNZ_LAYOUT_FOOTAGE_01</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>レイアウト</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>全画面映像＋キャラクター</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>render_verified</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>1.1.0</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>layouts/v1.1.0/manifest.json</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>共通素材</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>独自実装／既存共通演出再利用</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>validation/extension/qc-report.json</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>既存V02・旧EP・過去レンダーは不変</t>
+        </is>
+      </c>
+      <c r="K14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>NNZ_LAYOUT_DIAGRAM_01</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>レイアウト</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>全画面図解＋任意キャラクター</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>render_verified</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>1.1.0</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>layouts/v1.1.0/manifest.json</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>共通素材</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>独自実装／既存共通演出再利用</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>validation/extension/qc-report.json</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>既存V02・旧EP・過去レンダーは不変</t>
+        </is>
+      </c>
+      <c r="K15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>NNZ_LAYOUT_FOCUS_01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>レイアウト</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>実物→注目箇所拡大→断面→実物</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>render_verified</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>1.1.0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>layouts/v1.1.0/manifest.json</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>共通素材</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>独自実装／既存共通演出再利用</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>validation/extension/qc-report.json</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>既存V02・旧EP・過去レンダーは不変</t>
+        </is>
+      </c>
+      <c r="K16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>NNZ_TMP_LABEL_01</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>テンプレ</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>部分ラベルの順次表示</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>render_verified</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1.1.0</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>diagram_templates/label_01/1.1.0/manifest.json</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>共通素材</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>独自実装／既存共通演出再利用</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>validation/extension/qc-report.json</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>既存V02・旧EP・過去レンダーは不変</t>
+        </is>
+      </c>
+      <c r="K17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>NNZ_TMP_STEP3_01</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>テンプレ</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>3段階の因果説明</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>render_verified</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>1.1.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>diagram_templates/step3_01/1.1.0/manifest.json</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>共通素材</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>独自実装／既存共通演出再利用</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>validation/extension/qc-report.json</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>既存V02・旧EP・過去レンダーは不変</t>
+        </is>
+      </c>
+      <c r="K18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>NNZ_TMP_CROSSSECTION_01</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>テンプレ</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>物体に依存しない断面レイヤー</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>render_verified</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1.1.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>diagram_templates/crosssection_01/1.1.0/manifest.json</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>共通素材</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>独自実装／既存共通演出再利用</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>validation/extension/qc-report.json</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>既存V02・旧EP・過去レンダーは不変</t>
+        </is>
+      </c>
+      <c r="K19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>NNZ_MOTION_BASIC_01</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>動作</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>登場・退場・待機・うなずき・ポーズ切替</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>render_verified</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>1.1.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>animation/basic_01/1.1.0/manifest.json</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>共通素材</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>独自実装／既存共通演出再利用</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>validation/extension/qc-report.json</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>既存V02・旧EP・過去レンダーは不変</t>
+        </is>
+      </c>
+      <c r="K20" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:K20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Complete EP004 ice V3 cut assets and register reusable ice resources
</commit_message>
<xml_diff>
--- a/common_assets/nichijou_naze/management/asset_registry.xlsx
+++ b/common_assets/nichijou_naze/management/asset_registry.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Assets'!$A$1:$K$20</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -415,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1520,8 +1518,502 @@
         <v>1</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>NNZ_PROP_ICE_CLOUDY_PHOTO_01</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>photograph</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>家庭の白い氷 実写風</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>self_qc_render_verified</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>props/ice_v3/v1.0.0/manifest.json</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>EP004 V3</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Original AI reenactment / original Three.js geometry. See EP004_ICE_V3/licenses/. No official artwork reused.</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>EP004_ICE_V3/qc/full_v3/report.json</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>AI再現。中心の白濁。実験映像ではない。</t>
+        </is>
+      </c>
+      <c r="K21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>NNZ_PROP_ICE_PROCESS_PHOTO_01</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>photo_set</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>沸騰・冷却・注水の実写風セット</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>self_qc_render_verified</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>props/ice_v3/v1.0.0/manifest.json</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>EP004 V3</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Original AI reenactment / original Three.js geometry. See EP004_ICE_V3/licenses/. No official artwork reused.</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>EP004_ICE_V3/qc/full_v3/report.json</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>液体の工程。完成した透明氷は含まない。</t>
+        </is>
+      </c>
+      <c r="K22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>NNZ_PROP_ICE_CONDITION_PHOTO_01</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>photograph</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>条件による白濁量の例 実写風</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>self_qc_render_verified</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>props/ice_v3/v1.0.0/manifest.json</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>EP004 V3</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Original AI reenactment / original Three.js geometry. See EP004_ICE_V3/licenses/. No official artwork reused.</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>EP004_ICE_V3/qc/full_v3/report.json</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>沸騰後も白濁が残る一例。必ず白くなる意味ではない。</t>
+        </is>
+      </c>
+      <c r="K23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>NNZ_PROP_ICE_COMPARE_PHOTO_01</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>photograph</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>同条件の氷比較 実写風</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>self_qc_render_verified</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>props/ice_v3/v1.0.0/manifest.json</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>EP004 V3</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Original AI reenactment / original Three.js geometry. See EP004_ICE_V3/licenses/. No official artwork reused.</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>EP004_ICE_V3/qc/full_v3/report.json</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>左右同照明・同程度サイズ。白濁量は条件依存。</t>
+        </is>
+      </c>
+      <c r="K24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>NNZ_PROP_ICE_FACTORY_PHOTO_01</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>photograph</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>製氷工場 実写風</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>self_qc_render_verified</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>props/ice_v3/v1.0.0/manifest.json</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>EP004 V3</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Original AI reenactment / original Three.js geometry. See EP004_ICE_V3/licenses/. No official artwork reused.</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>EP004_ICE_V3/qc/full_v3/report.json</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>AI再現。公式工場写真ではない。</t>
+        </is>
+      </c>
+      <c r="K25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>NNZ_MODEL_ICE_MICRO_01</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Three.js scene</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>氷内部の気泡と光散乱</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>self_qc_render_verified</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>props/ice_v3/v1.0.0/manifest.json</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>EP004 V3</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Original AI reenactment / original Three.js geometry. See EP004_ICE_V3/licenses/. No official artwork reused.</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>EP004_ICE_V3/qc/full_v3/report.json</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>光線の分岐・泡の寸法は拡大模式。キャラクターと文字は別レイヤー。</t>
+        </is>
+      </c>
+      <c r="K26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>NNZ_MODEL_FREEZING_CELL_01</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Three.js scene</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>家庭の製氷皿 連続凍結断面</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>self_qc_render_verified</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>props/ice_v3/v1.0.0/manifest.json</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>EP004 V3</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Original AI reenactment / original Three.js geometry. See EP004_ICE_V3/licenses/. No official artwork reused.</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>EP004_ICE_V3/qc/full_v3/report.json</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>凍結形は模式。外側凍結→中心の気体集積→微細空洞。</t>
+        </is>
+      </c>
+      <c r="K27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>NNZ_MODEL_ICECAN_AIR_01</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Three.js scene</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>製氷缶 送気と遅い凍結</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>self_qc_render_verified</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>props/ice_v3/v1.0.0/manifest.json</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>EP004 V3</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Original AI reenactment / original Three.js geometry. See EP004_ICE_V3/licenses/. No official artwork reused.</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>EP004_ICE_V3/qc/full_v3/report.json</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>橙色管は送気。吸引ではない。中心の水を保持。</t>
+        </is>
+      </c>
+      <c r="K28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>NNZ_MODEL_ICECAN_DRAIN_01</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Three.js scene</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>製氷缶 中心液体の吸引</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>self_qc_render_verified</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>props/ice_v3/v1.0.0/manifest.json</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>EP004 V3</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Original AI reenactment / original Three.js geometry. See EP004_ICE_V3/licenses/. No official artwork reused.</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>EP004_ICE_V3/qc/full_v3/report.json</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>青色管は吸水。固体を削らない。中心液体と受器の体積保存。</t>
+        </is>
+      </c>
+      <c r="K29" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add verified reusable asset library operations and standalone EP reuse workflow
</commit_message>
<xml_diff>
--- a/common_assets/nichijou_naze/management/asset_registry.xlsx
+++ b/common_assets/nichijou_naze/management/asset_registry.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2013,6 +2013,226 @@
         <v>1</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>NNZ_MODEL_ICE_MICRO_01</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>氷内部の気泡と光散乱</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>self_qc_render_verified</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>1.1.0</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>common_assets/nichijou_naze/management/operations/v1/registrations/NNZ_MODEL_ICE_MICRO_01/1.1.0.json</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>EP004_ICE_V3 (extracted without changing original; import paths only)</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Original procedural geometry. Adapted from EP004; no copied manufacturer artwork. Three.js MIT. Scientific dimensions/timing are schematic.</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>validation/library-ops/reuse-model-qc.json</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Immutable standalone reusable version. domain</t>
+        </is>
+      </c>
+      <c r="K30" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>NNZ_MODEL_FREEZING_CELL_01</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>製氷皿の連続凍結断面</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>self_qc_render_verified</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1.1.0</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>common_assets/nichijou_naze/management/operations/v1/registrations/NNZ_MODEL_FREEZING_CELL_01/1.1.0.json</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>EP004_ICE_V3 (extracted without changing original; import paths only)</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Original procedural geometry. Adapted from EP004; no copied manufacturer artwork. Three.js MIT. Scientific dimensions/timing are schematic.</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>validation/library-ops/reuse-model-qc.json</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Immutable standalone reusable version. domain</t>
+        </is>
+      </c>
+      <c r="K31" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>NNZ_MODEL_ICECAN_AIR_01</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>製氷缶の送気と遅い凍結</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>self_qc_render_verified</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>1.1.0</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>common_assets/nichijou_naze/management/operations/v1/registrations/NNZ_MODEL_ICECAN_AIR_01/1.1.0.json</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>EP004_ICE_V3 (extracted without changing original; import paths only)</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Original procedural geometry. Adapted from EP004; no copied manufacturer artwork. Three.js MIT. Scientific dimensions/timing are schematic.</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>validation/library-ops/reuse-model-qc.json</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Immutable standalone reusable version. domain</t>
+        </is>
+      </c>
+      <c r="K32" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>NNZ_MODEL_ICECAN_DRAIN_01</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>製氷缶の中心液体吸引</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>self_qc_render_verified</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>1.1.0</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>common_assets/nichijou_naze/management/operations/v1/registrations/NNZ_MODEL_ICECAN_DRAIN_01/1.1.0.json</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>EP004_ICE_V3 (extracted without changing original; import paths only)</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Original procedural geometry. Adapted from EP004; no copied manufacturer artwork. Three.js MIT. Scientific dimensions/timing are schematic.</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>validation/library-ops/reuse-model-qc.json</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Immutable standalone reusable version. domain</t>
+        </is>
+      </c>
+      <c r="K33" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>